<commit_message>
+ added publication for smuLA26
</commit_message>
<xml_diff>
--- a/List of Kinetic Models.xlsx
+++ b/List of Kinetic Models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\MyProjects\kinmodre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC26B776-21EB-404E-A452-C70B8688A1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A9076E4-43C5-42A9-B0D3-4DAFF35A75F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A48245FD-6B6A-497E-8B16-C1CADEA3146F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="107">
   <si>
     <t>Model Name</t>
   </si>
@@ -522,6 +522,9 @@
   </si>
   <si>
     <t>Verma et al. 2026. Ab Initio Whole Cell Kinetic Model of Streptococcus thermophilus STH_CIRM_65 (stheVS26). Acta Scientific Nutritional Health 10(2): 43-47.</t>
+  </si>
+  <si>
+    <t>Cinco et al. 2026. Ab Initio Whole Cell Kinetic Model of Streptomyces murinus CR-43 (smuLA26). Journal of Clinical Immunology &amp; Microbiology 7(1): 1-5.</t>
   </si>
 </sst>
 </file>
@@ -1610,7 +1613,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>99</v>
       </c>
@@ -1631,6 +1634,9 @@
       </c>
       <c r="G26" s="2">
         <v>1009</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
+ added publication for blmSHM26
</commit_message>
<xml_diff>
--- a/List of Kinetic Models.xlsx
+++ b/List of Kinetic Models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\MyProjects\kinmodre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0227471-8000-4529-AE4F-4D7D49DA1882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{983BD7FF-7989-4A58-90E3-C6FFDF1D3E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A48245FD-6B6A-497E-8B16-C1CADEA3146F}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="129">
   <si>
     <t>Model Name</t>
   </si>
@@ -435,9 +435,6 @@
     <t>G9842</t>
   </si>
   <si>
-    <t>Ambel et al. 2025. UniKin2 – A Universal, Pan-Reactome Kinetic Model. International Journal of Research in Medical and Clinical Science 3(2): 77-80.</t>
-  </si>
-  <si>
     <t>spnLHP26</t>
   </si>
   <si>
@@ -592,6 +589,12 @@
   </si>
   <si>
     <t>bbrdPS26</t>
+  </si>
+  <si>
+    <t>Ambel et al. (2025) UniKin2 – A Universal, Pan-Reactome Kinetic Model. International Journal of Research in Medical and Clinical Science 3(2): 77-80.</t>
+  </si>
+  <si>
+    <t>Modankap et al. (2026) Ab Initio Whole Cell Kinetic Model of Bifidobacterium longum subsp. longum JCM1217 (blmSHM26). American Journal of Pathology &amp; Research 5(8): 1-5.</t>
   </si>
 </sst>
 </file>
@@ -1054,18 +1057,18 @@
   <sheetData>
     <row r="1" spans="1:2" s="8" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>111</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -1194,12 +1197,12 @@
         <v>701</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B4" s="2">
         <v>2026</v>
@@ -1208,7 +1211,7 @@
         <v>61</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E4" s="2">
         <v>752</v>
@@ -1220,7 +1223,7 @@
         <v>703</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="31" x14ac:dyDescent="0.35">
@@ -1277,16 +1280,16 @@
     </row>
     <row r="7" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B7" s="2">
         <v>2026</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E7" s="2">
         <v>861</v>
@@ -1298,12 +1301,12 @@
         <v>580</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B8" s="2">
         <v>2026</v>
@@ -1324,12 +1327,12 @@
         <v>846</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B9" s="2">
         <v>2026</v>
@@ -1350,21 +1353,21 @@
         <v>842</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B10" s="2">
         <v>2026</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>86</v>
       </c>
       <c r="E10" s="2">
         <v>1126</v>
@@ -1378,7 +1381,7 @@
     </row>
     <row r="11" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B11" s="2">
         <v>2026</v>
@@ -1399,12 +1402,12 @@
         <v>322</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B12" s="2">
         <v>2026</v>
@@ -1425,12 +1428,12 @@
         <v>1097</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B13" s="2">
         <v>2026</v>
@@ -1451,21 +1454,21 @@
         <v>919</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B14" s="2">
         <v>2026</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E14" s="2">
         <v>1385</v>
@@ -1477,7 +1480,7 @@
         <v>1009</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -1503,21 +1506,21 @@
         <v>1059</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B16" s="2">
         <v>2026</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="E16" s="2">
         <v>1153</v>
@@ -1529,12 +1532,12 @@
         <v>986</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17" s="2">
         <v>2026</v>
@@ -1555,12 +1558,12 @@
         <v>816</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B18" s="2">
         <v>2026</v>
@@ -1581,12 +1584,12 @@
         <v>1014</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B19" s="2">
         <v>2026</v>
@@ -1607,12 +1610,12 @@
         <v>1230</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B20" s="2">
         <v>2026</v>
@@ -1633,12 +1636,12 @@
         <v>802</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B21" s="2">
         <v>2026</v>
@@ -1659,7 +1662,7 @@
         <v>1208</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="31" x14ac:dyDescent="0.35">
@@ -1945,21 +1948,21 @@
         <v>30669</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B33" s="2">
         <v>2026</v>
       </c>
       <c r="C33" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="E33" s="2">
         <v>580</v>
@@ -1971,18 +1974,18 @@
         <v>453</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B34" s="2">
         <v>2026</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E34" s="2">
         <v>753</v>
@@ -1993,19 +1996,22 @@
       <c r="G34" s="2">
         <v>731</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H34" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B35" s="2">
         <v>2026</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E35" s="2">
         <v>1195</v>
@@ -2017,18 +2023,18 @@
         <v>1109</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B36" s="2">
         <v>2026</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E36" s="2">
         <v>1736</v>

</xml_diff>